<commit_message>
V1 van weggelaten woordgroepen
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/STAP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/STAP_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1A70C9-F124-49B0-A84D-CD8BFF599632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20076EFA-5917-4648-937A-BC978ADD9415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="245">
   <si>
     <t>Item</t>
   </si>
@@ -825,10 +825,13 @@
     <t>S060</t>
   </si>
   <si>
-    <t>opmerkingen</t>
-  </si>
-  <si>
     <t>get_pronunciation_variants</t>
+  </si>
+  <si>
+    <t>omitted_phrase</t>
+  </si>
+  <si>
+    <t>SASTA-opmerkingen</t>
   </si>
 </sst>
 </file>
@@ -2618,7 +2621,9 @@
       <c r="I37" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="L37" s="6"/>
+      <c r="L37" s="6" t="s">
+        <v>243</v>
+      </c>
       <c r="M37" s="2" t="s">
         <v>182</v>
       </c>
@@ -2744,7 +2749,7 @@
         <v>241</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>240</v>
@@ -2753,7 +2758,7 @@
         <v>158</v>
       </c>
       <c r="L42" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>182</v>

</xml_diff>

<commit_message>
del_nmwg en topic_drop updates
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/STAP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/STAP_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20076EFA-5917-4648-937A-BC978ADD9415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4909186-36D0-4AF6-BF4C-71B0EE73E15C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="247">
   <si>
     <t>Item</t>
   </si>
@@ -832,6 +832,12 @@
   </si>
   <si>
     <t>SASTA-opmerkingen</t>
+  </si>
+  <si>
+    <t>S061</t>
+  </si>
+  <si>
+    <t>topic_drop</t>
   </si>
 </sst>
 </file>
@@ -1842,7 +1848,7 @@
       <c r="K14" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="L14" s="6" t="s">
+      <c r="L14" s="2" t="s">
         <v>119</v>
       </c>
       <c r="M14" s="2" t="s">
@@ -1880,7 +1886,7 @@
       <c r="K15" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="L15" s="6"/>
+      <c r="L15" s="2"/>
       <c r="M15" s="2" t="s">
         <v>97</v>
       </c>
@@ -1916,7 +1922,7 @@
       <c r="K16" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="L16" s="6" t="s">
+      <c r="L16" s="2" t="s">
         <v>116</v>
       </c>
       <c r="M16" s="2" t="s">
@@ -1954,7 +1960,7 @@
       <c r="K17" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="L17" s="6" t="s">
+      <c r="L17" s="2" t="s">
         <v>117</v>
       </c>
       <c r="M17" s="2" t="s">
@@ -2059,7 +2065,7 @@
       <c r="H20" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="L20" s="2" t="s">
         <v>143</v>
       </c>
       <c r="M20" s="2" t="s">
@@ -2091,7 +2097,7 @@
       <c r="I21" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="L21" s="7" t="s">
+      <c r="L21" s="2" t="s">
         <v>157</v>
       </c>
       <c r="M21" s="2" t="s">
@@ -2126,7 +2132,7 @@
       <c r="I22" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="L22" s="7" t="s">
+      <c r="L22" s="2" t="s">
         <v>178</v>
       </c>
       <c r="M22" s="2" t="s">
@@ -2161,7 +2167,7 @@
       <c r="I23" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="L23" s="7" t="s">
+      <c r="L23" s="2" t="s">
         <v>168</v>
       </c>
       <c r="M23" s="2" t="s">
@@ -2193,7 +2199,7 @@
       <c r="H24" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="L24" s="7" t="s">
+      <c r="L24" s="2" t="s">
         <v>170</v>
       </c>
       <c r="M24" s="2" t="s">
@@ -2228,7 +2234,7 @@
       <c r="I25" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="L25" s="6" t="s">
+      <c r="L25" s="2" t="s">
         <v>174</v>
       </c>
       <c r="M25" s="2" t="s">
@@ -2263,7 +2269,7 @@
       <c r="I26" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="L26" s="6" t="s">
+      <c r="L26" s="2" t="s">
         <v>177</v>
       </c>
       <c r="M26" s="2" t="s">
@@ -2295,7 +2301,7 @@
       <c r="I27" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="L27" s="6" t="s">
+      <c r="L27" s="2" t="s">
         <v>181</v>
       </c>
       <c r="M27" s="2" t="s">
@@ -2330,7 +2336,7 @@
       <c r="I28" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="L28" s="6" t="s">
+      <c r="L28" s="2" t="s">
         <v>185</v>
       </c>
       <c r="M28" s="2" t="s">
@@ -2362,7 +2368,7 @@
       <c r="I29" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="L29" s="6" t="s">
+      <c r="L29" s="2" t="s">
         <v>194</v>
       </c>
       <c r="M29" s="2" t="s">
@@ -2394,7 +2400,7 @@
       <c r="I30" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="L30" s="6" t="s">
+      <c r="L30" s="2" t="s">
         <v>197</v>
       </c>
       <c r="M30" s="2" t="s">
@@ -2423,7 +2429,7 @@
       <c r="H31" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="L31" s="6" t="s">
+      <c r="L31" s="2" t="s">
         <v>200</v>
       </c>
       <c r="M31" s="2" t="s">
@@ -2455,7 +2461,7 @@
       <c r="H32" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="L32" s="6" t="s">
+      <c r="L32" s="2" t="s">
         <v>209</v>
       </c>
       <c r="M32" s="2" t="s">
@@ -2484,7 +2490,7 @@
       <c r="H33" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="L33" s="6" t="s">
+      <c r="L33" s="2" t="s">
         <v>208</v>
       </c>
       <c r="M33" s="2" t="s">
@@ -2519,7 +2525,7 @@
       <c r="I34" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="L34" s="6" t="s">
+      <c r="L34" s="2" t="s">
         <v>205</v>
       </c>
       <c r="M34" s="2" t="s">
@@ -2554,7 +2560,7 @@
       <c r="I35" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="L35" s="6" t="s">
+      <c r="L35" s="2" t="s">
         <v>213</v>
       </c>
       <c r="M35" s="2" t="s">
@@ -2589,7 +2595,7 @@
       <c r="I36" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="L36" s="6" t="s">
+      <c r="L36" s="2" t="s">
         <v>216</v>
       </c>
       <c r="M36" s="2" t="s">
@@ -2621,7 +2627,7 @@
       <c r="I37" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="L37" s="6" t="s">
+      <c r="L37" s="2" t="s">
         <v>243</v>
       </c>
       <c r="M37" s="2" t="s">
@@ -2650,7 +2656,7 @@
       <c r="I38" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="L38" s="6" t="s">
+      <c r="L38" s="2" t="s">
         <v>226</v>
       </c>
       <c r="M38" s="2" t="s">
@@ -2676,7 +2682,7 @@
       <c r="H39" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="L39" s="6" t="s">
+      <c r="L39" s="2" t="s">
         <v>229</v>
       </c>
       <c r="M39" s="2" t="s">
@@ -2705,7 +2711,7 @@
       <c r="I40" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="L40" s="6" t="s">
+      <c r="L40" s="2" t="s">
         <v>233</v>
       </c>
       <c r="M40" s="2" t="s">
@@ -2731,7 +2737,7 @@
       <c r="H41" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="L41" s="6" t="s">
+      <c r="L41" s="2" t="s">
         <v>239</v>
       </c>
       <c r="M41" s="2" t="s">
@@ -2757,7 +2763,7 @@
       <c r="H42" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="L42" s="7" t="s">
+      <c r="L42" s="2" t="s">
         <v>242</v>
       </c>
       <c r="M42" s="2" t="s">
@@ -2767,6 +2773,26 @@
         <v>158</v>
       </c>
       <c r="O42" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="O43" s="2" t="s">
         <v>104</v>
       </c>
     </row>

</xml_diff>

<commit_message>
false start, self correction, repetition counts added
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/STAP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/STAP_Index_Current.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAAE0D88-0712-46FE-855A-863036CF4679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980A661F-B594-4D53-A1EA-F4FB7FEEA68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="260">
   <si>
     <t>Item</t>
   </si>
@@ -838,6 +838,45 @@
   </si>
   <si>
     <t>topic_drop</t>
+  </si>
+  <si>
+    <t>S062</t>
+  </si>
+  <si>
+    <t>valse_start</t>
+  </si>
+  <si>
+    <t>valse start</t>
+  </si>
+  <si>
+    <t>62-63</t>
+  </si>
+  <si>
+    <t>false_start</t>
+  </si>
+  <si>
+    <t>S063</t>
+  </si>
+  <si>
+    <t>zelfverbetering</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>self_correction</t>
+  </si>
+  <si>
+    <t>S064</t>
+  </si>
+  <si>
+    <t>herhaling</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>repetition</t>
   </si>
 </sst>
 </file>
@@ -2792,39 +2831,126 @@
       <c r="L43" s="2" t="s">
         <v>246</v>
       </c>
+      <c r="M43" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>158</v>
+      </c>
       <c r="O43" s="2" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="44" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="L44" s="6"/>
+      <c r="A44" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N44" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O44" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="45" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="L45" s="6"/>
+      <c r="A45" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O45" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="46" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="L46" s="6"/>
+      <c r="A46" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="M46" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N46" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O46" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="47" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="L47" s="6"/>
+      <c r="L47" s="2"/>
     </row>
     <row r="48" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="L48" s="6"/>
+      <c r="L48" s="2"/>
     </row>
     <row r="49" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L49" s="6"/>
+      <c r="L49" s="2"/>
     </row>
     <row r="50" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L50" s="6"/>
+      <c r="L50" s="2"/>
     </row>
     <row r="51" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L51" s="6"/>
+      <c r="L51" s="2"/>
     </row>
     <row r="52" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L52" s="6"/>
+      <c r="L52" s="2"/>
     </row>
     <row r="53" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L53" s="6"/>
+      <c r="L53" s="2"/>
     </row>
     <row r="54" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L54" s="6"/>

</xml_diff>

<commit_message>
Improved silver data and improved permcomments
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/STAP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/STAP_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980A661F-B594-4D53-A1EA-F4FB7FEEA68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75423EB-C9CB-4136-8D89-9EA567D20184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="263">
   <si>
     <t>Item</t>
   </si>
@@ -750,9 +750,6 @@
     <t>verb_no_pv</t>
   </si>
   <si>
-    <t>bep deletie</t>
-  </si>
-  <si>
     <t>S036</t>
   </si>
   <si>
@@ -877,6 +874,18 @@
   </si>
   <si>
     <t>repetition</t>
+  </si>
+  <si>
+    <t>uitspraak-variant, uitspraakvariant, uitspraak variant</t>
+  </si>
+  <si>
+    <t>beginwoorddeletie</t>
+  </si>
+  <si>
+    <t>topic_drop, bw_del, bwd</t>
+  </si>
+  <si>
+    <t>bep deletie, bepaler_weg</t>
   </si>
 </sst>
 </file>
@@ -2128,7 +2137,7 @@
         <v>156</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>217</v>
+        <v>262</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>97</v>
@@ -2367,7 +2376,7 @@
         <v>184</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>97</v>
@@ -2495,7 +2504,7 @@
         <v>206</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>158</v>
@@ -2556,7 +2565,7 @@
         <v>204</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>97</v>
@@ -2623,10 +2632,10 @@
         <v>165</v>
       </c>
       <c r="E36" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>235</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>236</v>
       </c>
       <c r="H36" s="2" t="s">
         <v>97</v>
@@ -2649,25 +2658,25 @@
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>165</v>
       </c>
       <c r="E37" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="F37" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="F37" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="H37" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="M37" s="2" t="s">
         <v>182</v>
@@ -2681,13 +2690,13 @@
     </row>
     <row r="38" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>165</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>97</v>
@@ -2696,7 +2705,7 @@
         <v>187</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="M38" s="2" t="s">
         <v>182</v>
@@ -2710,19 +2719,19 @@
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>165</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>97</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="M39" s="2" t="s">
         <v>182</v>
@@ -2736,22 +2745,22 @@
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>165</v>
       </c>
       <c r="E40" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I40" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="H40" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I40" s="2" t="s">
+      <c r="L40" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="L40" s="2" t="s">
-        <v>233</v>
       </c>
       <c r="M40" s="2" t="s">
         <v>182</v>
@@ -2765,19 +2774,19 @@
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D41" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="L41" s="2" t="s">
         <v>238</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>239</v>
       </c>
       <c r="M41" s="2" t="s">
         <v>182</v>
@@ -2791,19 +2800,22 @@
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>259</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>158</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="M42" s="2" t="s">
         <v>182</v>
@@ -2817,19 +2829,22 @@
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>246</v>
+        <v>260</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>261</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>158</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="M43" s="2" t="s">
         <v>182</v>
@@ -2843,25 +2858,25 @@
     </row>
     <row r="44" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="E44" s="2" t="s">
+      <c r="F44" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="H44" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I44" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="H44" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I44" s="2" t="s">
+      <c r="L44" s="2" t="s">
         <v>250</v>
-      </c>
-      <c r="L44" s="2" t="s">
-        <v>251</v>
       </c>
       <c r="M44" s="2" t="s">
         <v>182</v>
@@ -2875,22 +2890,22 @@
     </row>
     <row r="45" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="E45" s="2" t="s">
+      <c r="H45" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I45" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="H45" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I45" s="2" t="s">
+      <c r="L45" s="2" t="s">
         <v>254</v>
-      </c>
-      <c r="L45" s="2" t="s">
-        <v>255</v>
       </c>
       <c r="M45" s="2" t="s">
         <v>182</v>
@@ -2904,22 +2919,22 @@
     </row>
     <row r="46" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E46" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="E46" s="2" t="s">
+      <c r="H46" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I46" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="H46" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I46" s="2" t="s">
+      <c r="L46" s="2" t="s">
         <v>258</v>
-      </c>
-      <c r="L46" s="2" t="s">
-        <v>259</v>
       </c>
       <c r="M46" s="2" t="s">
         <v>182</v>

</xml_diff>

<commit_message>
aux_lexicons, stap form improvements, stap errors
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/STAP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/STAP_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75423EB-C9CB-4136-8D89-9EA567D20184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B1BDBC-7DC9-44E8-9920-2AAB39DCB1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$X$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$X$157</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="300">
   <si>
     <t>Item</t>
   </si>
@@ -887,12 +887,123 @@
   <si>
     <t>bep deletie, bepaler_weg</t>
   </si>
+  <si>
+    <t>S065</t>
+  </si>
+  <si>
+    <t>t_elisie</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>pv_t_elisions</t>
+  </si>
+  <si>
+    <t>t-elisie, t elisie</t>
+  </si>
+  <si>
+    <t>S041</t>
+  </si>
+  <si>
+    <t>S042</t>
+  </si>
+  <si>
+    <t>variabele 13</t>
+  </si>
+  <si>
+    <t>variabele 14</t>
+  </si>
+  <si>
+    <t>grammaticale fouten</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>S043</t>
+  </si>
+  <si>
+    <t>variabele 15</t>
+  </si>
+  <si>
+    <t>vt_fout_count</t>
+  </si>
+  <si>
+    <t>congruentie_fount_count</t>
+  </si>
+  <si>
+    <t>S044</t>
+  </si>
+  <si>
+    <t>variabele 16</t>
+  </si>
+  <si>
+    <t>vd_fout_count</t>
+  </si>
+  <si>
+    <t>S045</t>
+  </si>
+  <si>
+    <t>variabele 17</t>
+  </si>
+  <si>
+    <t>nmwg_weg_count</t>
+  </si>
+  <si>
+    <t>S046</t>
+  </si>
+  <si>
+    <t>variabele 18</t>
+  </si>
+  <si>
+    <t>bepaler_weg_count</t>
+  </si>
+  <si>
+    <t>S047</t>
+  </si>
+  <si>
+    <t>variabele 19</t>
+  </si>
+  <si>
+    <t>S048</t>
+  </si>
+  <si>
+    <t>variabele 20</t>
+  </si>
+  <si>
+    <t>woordvolgordefout_count</t>
+  </si>
+  <si>
+    <t>S049</t>
+  </si>
+  <si>
+    <t>ov:uiting_count</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>congruentie_fouten_count</t>
+  </si>
+  <si>
+    <t>bepaler_verkeerd_count</t>
+  </si>
+  <si>
+    <t>ov_uiting_count</t>
+  </si>
+  <si>
+    <t>del_nmwg_count</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -920,6 +1031,12 @@
       <color theme="1"/>
       <name val="Courier New"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1314,7 +1431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X149"/>
+  <dimension ref="A1:X158"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.77734375" style="2"/>
@@ -2800,23 +2917,18 @@
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>259</v>
+        <v>268</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>270</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>241</v>
-      </c>
+        <v>97</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="L42" s="2"/>
       <c r="M42" s="2" t="s">
         <v>182</v>
       </c>
@@ -2824,27 +2936,30 @@
         <v>158</v>
       </c>
       <c r="O42" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>244</v>
+        <v>269</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>271</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>261</v>
+        <v>277</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>158</v>
+        <v>97</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>273</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>245</v>
+        <v>296</v>
       </c>
       <c r="M43" s="2" t="s">
         <v>182</v>
@@ -2853,30 +2968,30 @@
         <v>158</v>
       </c>
       <c r="O43" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="44" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>246</v>
+        <v>274</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>275</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>248</v>
+        <v>276</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>249</v>
+        <v>294</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="M44" s="2" t="s">
         <v>182</v>
@@ -2885,27 +3000,30 @@
         <v>158</v>
       </c>
       <c r="O44" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="45" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>251</v>
+        <v>278</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>279</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>252</v>
+        <v>280</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>253</v>
+        <v>215</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>254</v>
+        <v>280</v>
       </c>
       <c r="M45" s="2" t="s">
         <v>182</v>
@@ -2914,27 +3032,30 @@
         <v>158</v>
       </c>
       <c r="O45" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="46" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>255</v>
+        <v>281</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>282</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>256</v>
+        <v>283</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>257</v>
+        <v>190</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>258</v>
+        <v>299</v>
       </c>
       <c r="M46" s="2" t="s">
         <v>182</v>
@@ -2943,56 +3064,332 @@
         <v>158</v>
       </c>
       <c r="O46" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="M47" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N47" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O47" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="M48" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O48" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="L49" s="2"/>
+      <c r="M49" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N49" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O49" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="M50" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O50" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="M51" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O51" s="2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="L47" s="2"/>
-    </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="L48" s="2"/>
-    </row>
-    <row r="49" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L49" s="2"/>
-    </row>
-    <row r="50" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L50" s="2"/>
-    </row>
-    <row r="51" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L51" s="2"/>
-    </row>
-    <row r="52" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L52" s="2"/>
-    </row>
-    <row r="53" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L53" s="2"/>
-    </row>
-    <row r="54" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L54" s="6"/>
-    </row>
-    <row r="56" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L56" s="6"/>
-    </row>
-    <row r="57" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L57" s="6"/>
-    </row>
-    <row r="58" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L58" s="6"/>
-    </row>
-    <row r="59" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L59" s="6"/>
-    </row>
-    <row r="60" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L60" s="6"/>
-    </row>
-    <row r="61" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L61" s="6"/>
-    </row>
-    <row r="63" spans="12:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="L52" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="M52" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N52" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O52" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="M53" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N53" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O53" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="M54" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O54" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="M55" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N55" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O55" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="M56" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N56" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O56" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L57" s="2"/>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L58" s="2"/>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L59" s="2"/>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L60" s="2"/>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L61" s="2"/>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L62" s="2"/>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="L63" s="6"/>
-    </row>
-    <row r="64" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L64" s="6"/>
     </row>
     <row r="65" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L65" s="6"/>
@@ -3003,6 +3400,9 @@
     <row r="67" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L67" s="6"/>
     </row>
+    <row r="68" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L68" s="6"/>
+    </row>
     <row r="69" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L69" s="6"/>
     </row>
@@ -3024,18 +3424,12 @@
     <row r="76" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L76" s="6"/>
     </row>
-    <row r="77" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L77" s="6"/>
-    </row>
     <row r="78" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L78" s="6"/>
     </row>
     <row r="79" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L79" s="6"/>
     </row>
-    <row r="80" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L80" s="6"/>
-    </row>
     <row r="81" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L81" s="6"/>
     </row>
@@ -3054,6 +3448,9 @@
     <row r="86" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L86" s="6"/>
     </row>
+    <row r="87" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L87" s="6"/>
+    </row>
     <row r="88" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L88" s="6"/>
     </row>
@@ -3072,15 +3469,21 @@
     <row r="93" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L93" s="6"/>
     </row>
+    <row r="94" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L94" s="6"/>
+    </row>
     <row r="95" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L95" s="6"/>
     </row>
-    <row r="96" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L96" s="6"/>
-    </row>
     <row r="97" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L97" s="6"/>
     </row>
+    <row r="98" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L98" s="6"/>
+    </row>
+    <row r="99" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L99" s="6"/>
+    </row>
     <row r="100" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L100" s="6"/>
     </row>
@@ -3090,119 +3493,138 @@
     <row r="102" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L102" s="6"/>
     </row>
-    <row r="103" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L103" s="6"/>
-    </row>
     <row r="104" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L104" s="6"/>
     </row>
-    <row r="107" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L107" s="6"/>
-    </row>
-    <row r="108" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L108" s="6"/>
+    <row r="105" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L105" s="6"/>
+    </row>
+    <row r="106" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L106" s="6"/>
+    </row>
+    <row r="109" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L109" s="6"/>
+    </row>
+    <row r="110" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L110" s="6"/>
+    </row>
+    <row r="111" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L111" s="6"/>
+    </row>
+    <row r="112" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L112" s="6"/>
     </row>
     <row r="113" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L113" s="6"/>
     </row>
-    <row r="114" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L114" s="6"/>
-    </row>
-    <row r="115" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L115" s="6"/>
-    </row>
     <row r="116" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L116" s="8"/>
+      <c r="L116" s="6"/>
     </row>
     <row r="117" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L117" s="6"/>
     </row>
-    <row r="118" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L118" s="6"/>
-    </row>
-    <row r="119" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L119" s="6"/>
-    </row>
-    <row r="120" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L120" s="6"/>
-    </row>
-    <row r="121" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L121" s="6"/>
-    </row>
     <row r="122" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L122" s="6"/>
     </row>
     <row r="123" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L123" s="6"/>
     </row>
+    <row r="124" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L124" s="6"/>
+    </row>
+    <row r="125" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L125" s="8"/>
+    </row>
+    <row r="126" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L126" s="6"/>
+    </row>
     <row r="127" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L127" s="6"/>
     </row>
     <row r="128" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L128" s="6"/>
     </row>
-    <row r="129" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="129" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L129" s="6"/>
     </row>
-    <row r="130" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="130" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L130" s="6"/>
     </row>
-    <row r="131" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="131" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L131" s="6"/>
     </row>
-    <row r="132" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="132" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L132" s="6"/>
     </row>
-    <row r="133" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="L133" s="6"/>
-    </row>
-    <row r="134" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="L134" s="6"/>
-    </row>
-    <row r="135" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="L135" s="6"/>
-    </row>
-    <row r="136" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="136" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L136" s="6"/>
     </row>
-    <row r="137" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="137" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L137" s="6"/>
     </row>
-    <row r="138" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="E138" s="3"/>
+    <row r="138" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L138" s="6"/>
     </row>
-    <row r="139" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="E139" s="3"/>
+    <row r="139" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L139" s="6"/>
     </row>
-    <row r="140" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="E140" s="4"/>
-    </row>
-    <row r="141" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="140" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L140" s="6"/>
+    </row>
+    <row r="141" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L141" s="6"/>
     </row>
-    <row r="143" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="142" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L142" s="6"/>
+    </row>
+    <row r="143" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L143" s="6"/>
     </row>
-    <row r="145" spans="12:12" x14ac:dyDescent="0.3">
+    <row r="144" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L144" s="6"/>
+    </row>
+    <row r="145" spans="5:12" x14ac:dyDescent="0.3">
       <c r="L145" s="6"/>
     </row>
-    <row r="147" spans="12:12" x14ac:dyDescent="0.3">
+    <row r="146" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L146" s="6"/>
+    </row>
+    <row r="147" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="E147" s="3"/>
       <c r="L147" s="6"/>
     </row>
-    <row r="148" spans="12:12" x14ac:dyDescent="0.3">
+    <row r="148" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="E148" s="3"/>
       <c r="L148" s="6"/>
     </row>
-    <row r="149" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L149" s="6"/>
+    <row r="149" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="E149" s="4"/>
+    </row>
+    <row r="150" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L150" s="6"/>
+    </row>
+    <row r="152" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L152" s="6"/>
+    </row>
+    <row r="154" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L154" s="6"/>
+    </row>
+    <row r="156" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L156" s="6"/>
+    </row>
+    <row r="157" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L157" s="6"/>
+    </row>
+    <row r="158" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L158" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X148" xr:uid="{FEE5544A-5DEE-468C-AA79-13446D744343}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N148">
-    <sortCondition ref="E2:E148"/>
-    <sortCondition ref="I2:I148"/>
+  <autoFilter ref="A1:X157" xr:uid="{FEE5544A-5DEE-468C-AA79-13446D744343}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N157">
+    <sortCondition ref="E2:E157"/>
+    <sortCondition ref="I2:I157"/>
   </sortState>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
improved table_comparison for grammatical errors
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/STAP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/STAP_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B1BDBC-7DC9-44E8-9920-2AAB39DCB1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7BDBE8-1391-4D48-9107-01B1222504EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$X$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$X$158</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="315">
   <si>
     <t>Item</t>
   </si>
@@ -762,9 +762,6 @@
     <t>deletie voorzetsel</t>
   </si>
   <si>
-    <t>deletie /er/</t>
-  </si>
-  <si>
     <t>deletie voegwrd</t>
   </si>
   <si>
@@ -810,9 +807,6 @@
     <t>sub_lexicaal</t>
   </si>
   <si>
-    <t>semantische fout</t>
-  </si>
-  <si>
     <t>sub_lexical</t>
   </si>
   <si>
@@ -915,9 +909,6 @@
     <t>variabele 14</t>
   </si>
   <si>
-    <t>grammaticale fouten</t>
-  </si>
-  <si>
     <t>39</t>
   </si>
   <si>
@@ -997,6 +988,60 @@
   </si>
   <si>
     <t>del_nmwg_count</t>
+  </si>
+  <si>
+    <t>S050</t>
+  </si>
+  <si>
+    <t>hoofdww weg</t>
+  </si>
+  <si>
+    <t>hoofdww_weg</t>
+  </si>
+  <si>
+    <t>hoofdww_weg_count</t>
+  </si>
+  <si>
+    <t>hoofdww_weg,hoofdww-weg</t>
+  </si>
+  <si>
+    <t>deletie /er/, ov:del-er</t>
+  </si>
+  <si>
+    <t>ov:sub-vg</t>
+  </si>
+  <si>
+    <t>ov:sub-tijd</t>
+  </si>
+  <si>
+    <t>sub-lexicaal</t>
+  </si>
+  <si>
+    <t>ov:sub-vnw</t>
+  </si>
+  <si>
+    <t>ov:sub-bw</t>
+  </si>
+  <si>
+    <t>ov:del-bw</t>
+  </si>
+  <si>
+    <t>ov:sub-vz</t>
+  </si>
+  <si>
+    <t>dan-toen-fout</t>
+  </si>
+  <si>
+    <t>adj-congr-fout</t>
+  </si>
+  <si>
+    <t>bbp</t>
+  </si>
+  <si>
+    <t>bbt</t>
+  </si>
+  <si>
+    <t>bbo</t>
   </si>
 </sst>
 </file>
@@ -1431,7 +1476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X158"/>
+  <dimension ref="A1:X159"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.77734375" style="2"/>
@@ -1890,6 +1935,9 @@
       <c r="E11" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="F11" s="2" t="s">
+        <v>312</v>
+      </c>
       <c r="H11" s="2" t="s">
         <v>97</v>
       </c>
@@ -1928,6 +1976,9 @@
       <c r="E12" s="2" t="s">
         <v>89</v>
       </c>
+      <c r="F12" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="H12" s="2" t="s">
         <v>97</v>
       </c>
@@ -1966,6 +2017,9 @@
       <c r="E13" s="2" t="s">
         <v>83</v>
       </c>
+      <c r="F13" s="2" t="s">
+        <v>314</v>
+      </c>
       <c r="H13" s="2" t="s">
         <v>97</v>
       </c>
@@ -2254,7 +2308,7 @@
         <v>156</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>97</v>
@@ -2460,6 +2514,9 @@
       <c r="E27" s="2" t="s">
         <v>180</v>
       </c>
+      <c r="F27" s="2" t="s">
+        <v>309</v>
+      </c>
       <c r="H27" s="2" t="s">
         <v>97</v>
       </c>
@@ -2527,6 +2584,9 @@
       <c r="E29" s="2" t="s">
         <v>193</v>
       </c>
+      <c r="F29" s="2" t="s">
+        <v>308</v>
+      </c>
       <c r="H29" s="2" t="s">
         <v>97</v>
       </c>
@@ -2559,6 +2619,9 @@
       <c r="E30" s="2" t="s">
         <v>196</v>
       </c>
+      <c r="F30" s="2" t="s">
+        <v>307</v>
+      </c>
       <c r="H30" s="2" t="s">
         <v>97</v>
       </c>
@@ -2591,6 +2654,9 @@
       <c r="E31" s="2" t="s">
         <v>199</v>
       </c>
+      <c r="F31" s="2" t="s">
+        <v>306</v>
+      </c>
       <c r="H31" s="2" t="s">
         <v>158</v>
       </c>
@@ -2621,7 +2687,7 @@
         <v>206</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>158</v>
@@ -2652,6 +2718,9 @@
       <c r="E33" s="2" t="s">
         <v>207</v>
       </c>
+      <c r="F33" s="2" t="s">
+        <v>303</v>
+      </c>
       <c r="H33" s="2" t="s">
         <v>158</v>
       </c>
@@ -2682,7 +2751,7 @@
         <v>204</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>221</v>
+        <v>302</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>97</v>
@@ -2749,10 +2818,10 @@
         <v>165</v>
       </c>
       <c r="E36" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>234</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>235</v>
       </c>
       <c r="H36" s="2" t="s">
         <v>97</v>
@@ -2790,10 +2859,10 @@
         <v>97</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="M37" s="2" t="s">
         <v>182</v>
@@ -2807,13 +2876,16 @@
     </row>
     <row r="38" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>165</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>311</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>97</v>
@@ -2822,7 +2894,7 @@
         <v>187</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="M38" s="2" t="s">
         <v>182</v>
@@ -2836,19 +2908,22 @@
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>165</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>310</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>97</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="M39" s="2" t="s">
         <v>182</v>
@@ -2862,22 +2937,25 @@
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>165</v>
       </c>
       <c r="E40" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I40" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="H40" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I40" s="2" t="s">
+      <c r="L40" s="2" t="s">
         <v>231</v>
-      </c>
-      <c r="L40" s="2" t="s">
-        <v>232</v>
       </c>
       <c r="M40" s="2" t="s">
         <v>182</v>
@@ -2891,19 +2969,22 @@
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>237</v>
+        <v>165</v>
       </c>
       <c r="E41" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="L41" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>238</v>
       </c>
       <c r="M41" s="2" t="s">
         <v>182</v>
@@ -2917,18 +2998,26 @@
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="D42" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I42" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="H42" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I42" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="L42" s="2"/>
+      <c r="L42" s="2" t="s">
+        <v>300</v>
+      </c>
       <c r="M42" s="2" t="s">
         <v>182</v>
       </c>
@@ -2941,25 +3030,25 @@
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="B43" s="2" t="s">
-        <v>271</v>
-      </c>
       <c r="D43" s="2" t="s">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="M43" s="2" t="s">
         <v>182</v>
@@ -2973,25 +3062,25 @@
     </row>
     <row r="44" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="M44" s="2" t="s">
         <v>182</v>
@@ -3005,16 +3094,16 @@
     </row>
     <row r="45" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>97</v>
@@ -3023,7 +3112,7 @@
         <v>215</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="M45" s="2" t="s">
         <v>182</v>
@@ -3037,16 +3126,16 @@
     </row>
     <row r="46" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>97</v>
@@ -3055,7 +3144,7 @@
         <v>190</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="M46" s="2" t="s">
         <v>182</v>
@@ -3069,16 +3158,16 @@
     </row>
     <row r="47" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>97</v>
@@ -3087,7 +3176,7 @@
         <v>189</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="M47" s="2" t="s">
         <v>182</v>
@@ -3101,25 +3190,25 @@
     </row>
     <row r="48" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="M48" s="2" t="s">
         <v>182</v>
@@ -3133,16 +3222,16 @@
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="H49" s="2" t="s">
         <v>97</v>
@@ -3163,13 +3252,13 @@
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="H50" s="2" t="s">
         <v>97</v>
@@ -3178,7 +3267,7 @@
         <v>186</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="M50" s="2" t="s">
         <v>182</v>
@@ -3192,22 +3281,25 @@
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>240</v>
+        <v>297</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>243</v>
+        <v>165</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>239</v>
+        <v>298</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>259</v>
+        <v>301</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>158</v>
+        <v>97</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>291</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>241</v>
+        <v>299</v>
       </c>
       <c r="M51" s="2" t="s">
         <v>182</v>
@@ -3221,22 +3313,22 @@
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>260</v>
+        <v>237</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>158</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="M52" s="2" t="s">
         <v>182</v>
@@ -3250,25 +3342,22 @@
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D53" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="L53" s="2" t="s">
         <v>243</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I53" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="L53" s="2" t="s">
-        <v>250</v>
       </c>
       <c r="M53" s="2" t="s">
         <v>182</v>
@@ -3282,22 +3371,25 @@
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>252</v>
+        <v>245</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>246</v>
       </c>
       <c r="H54" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="M54" s="2" t="s">
         <v>182</v>
@@ -3311,22 +3403,22 @@
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="M55" s="2" t="s">
         <v>182</v>
@@ -3340,25 +3432,22 @@
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="M56" s="2" t="s">
         <v>182</v>
@@ -3371,7 +3460,36 @@
       </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="L57" s="2"/>
+      <c r="A57" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="L57" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="M57" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="N57" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="O57" s="2" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="L58" s="2"/>
@@ -3389,10 +3507,10 @@
       <c r="L62" s="2"/>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="L63" s="6"/>
-    </row>
-    <row r="65" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L65" s="6"/>
+      <c r="L63" s="2"/>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="L64" s="6"/>
     </row>
     <row r="66" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L66" s="6"/>
@@ -3409,8 +3527,8 @@
     <row r="70" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L70" s="6"/>
     </row>
-    <row r="72" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L72" s="6"/>
+    <row r="71" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L71" s="6"/>
     </row>
     <row r="73" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L73" s="6"/>
@@ -3424,14 +3542,14 @@
     <row r="76" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L76" s="6"/>
     </row>
-    <row r="78" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L78" s="6"/>
+    <row r="77" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L77" s="6"/>
     </row>
     <row r="79" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L79" s="6"/>
     </row>
-    <row r="81" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L81" s="6"/>
+    <row r="80" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L80" s="6"/>
     </row>
     <row r="82" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L82" s="6"/>
@@ -3475,8 +3593,8 @@
     <row r="95" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L95" s="6"/>
     </row>
-    <row r="97" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L97" s="6"/>
+    <row r="96" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L96" s="6"/>
     </row>
     <row r="98" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L98" s="6"/>
@@ -3493,8 +3611,8 @@
     <row r="102" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L102" s="6"/>
     </row>
-    <row r="104" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L104" s="6"/>
+    <row r="103" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L103" s="6"/>
     </row>
     <row r="105" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L105" s="6"/>
@@ -3502,8 +3620,8 @@
     <row r="106" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L106" s="6"/>
     </row>
-    <row r="109" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L109" s="6"/>
+    <row r="107" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L107" s="6"/>
     </row>
     <row r="110" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L110" s="6"/>
@@ -3517,14 +3635,14 @@
     <row r="113" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L113" s="6"/>
     </row>
-    <row r="116" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L116" s="6"/>
+    <row r="114" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L114" s="6"/>
     </row>
     <row r="117" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L117" s="6"/>
     </row>
-    <row r="122" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L122" s="6"/>
+    <row r="118" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L118" s="6"/>
     </row>
     <row r="123" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L123" s="6"/>
@@ -3533,10 +3651,10 @@
       <c r="L124" s="6"/>
     </row>
     <row r="125" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L125" s="8"/>
+      <c r="L125" s="6"/>
     </row>
     <row r="126" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L126" s="6"/>
+      <c r="L126" s="8"/>
     </row>
     <row r="127" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L127" s="6"/>
@@ -3556,8 +3674,8 @@
     <row r="132" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L132" s="6"/>
     </row>
-    <row r="136" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L136" s="6"/>
+    <row r="133" spans="12:12" x14ac:dyDescent="0.3">
+      <c r="L133" s="6"/>
     </row>
     <row r="137" spans="12:12" x14ac:dyDescent="0.3">
       <c r="L137" s="6"/>
@@ -3590,7 +3708,6 @@
       <c r="L146" s="6"/>
     </row>
     <row r="147" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="E147" s="3"/>
       <c r="L147" s="6"/>
     </row>
     <row r="148" spans="5:12" x14ac:dyDescent="0.3">
@@ -3598,19 +3715,20 @@
       <c r="L148" s="6"/>
     </row>
     <row r="149" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="E149" s="4"/>
+      <c r="E149" s="3"/>
+      <c r="L149" s="6"/>
     </row>
     <row r="150" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="L150" s="6"/>
-    </row>
-    <row r="152" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="L152" s="6"/>
-    </row>
-    <row r="154" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="L154" s="6"/>
-    </row>
-    <row r="156" spans="5:12" x14ac:dyDescent="0.3">
-      <c r="L156" s="6"/>
+      <c r="E150" s="4"/>
+    </row>
+    <row r="151" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L151" s="6"/>
+    </row>
+    <row r="153" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L153" s="6"/>
+    </row>
+    <row r="155" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L155" s="6"/>
     </row>
     <row r="157" spans="5:12" x14ac:dyDescent="0.3">
       <c r="L157" s="6"/>
@@ -3618,11 +3736,14 @@
     <row r="158" spans="5:12" x14ac:dyDescent="0.3">
       <c r="L158" s="6"/>
     </row>
+    <row r="159" spans="5:12" x14ac:dyDescent="0.3">
+      <c r="L159" s="6"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:X157" xr:uid="{FEE5544A-5DEE-468C-AA79-13446D744343}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N157">
-    <sortCondition ref="E2:E157"/>
-    <sortCondition ref="I2:I157"/>
+  <autoFilter ref="A1:X158" xr:uid="{FEE5544A-5DEE-468C-AA79-13446D744343}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N158">
+    <sortCondition ref="E2:E158"/>
+    <sortCondition ref="I2:I158"/>
   </sortState>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
mijne mijnes xxx S020 improvements
</commit_message>
<xml_diff>
--- a/src/sastadev/data/methods/STAP_Index_Current.xlsx
+++ b/src/sastadev/data/methods/STAP_Index_Current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\jodijk\myprograms\python\sastacode\mysastadev\src\sastadev\data\methods\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF94ED8-66BD-40BF-84A8-8893C17A105C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBBC223C-E4FC-4532-BDB5-F86E7F8F407E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -552,502 +552,503 @@
        ]</t>
   </si>
   <si>
+    <t xml:space="preserve">//node[%STAP_OS%]
+</t>
+  </si>
+  <si>
+    <t>S020</t>
+  </si>
+  <si>
+    <t>bepaler weg</t>
+  </si>
+  <si>
+    <t>get_missing_det</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>pages2005</t>
+  </si>
+  <si>
+    <t>pages2017</t>
+  </si>
+  <si>
+    <t>acq_order</t>
+  </si>
+  <si>
+    <t>implied_by</t>
+  </si>
+  <si>
+    <t>S021</t>
+  </si>
+  <si>
+    <t>bepaler fout</t>
+  </si>
+  <si>
+    <t>grammaticale fout</t>
+  </si>
+  <si>
+    <t>S022</t>
+  </si>
+  <si>
+    <t>congruentiefout</t>
+  </si>
+  <si>
+    <t>stap_congruentiefout</t>
+  </si>
+  <si>
+    <t>S023</t>
+  </si>
+  <si>
+    <t>pv_regionale_vorm</t>
+  </si>
+  <si>
+    <t>bepalers</t>
+  </si>
+  <si>
+    <t>congruentie</t>
+  </si>
+  <si>
+    <t>S024</t>
+  </si>
+  <si>
+    <t>vt_fout</t>
+  </si>
+  <si>
+    <t>morfologie</t>
+  </si>
+  <si>
+    <t>S025</t>
+  </si>
+  <si>
+    <t>vd_fout</t>
+  </si>
+  <si>
+    <t>stap_sublid</t>
+  </si>
+  <si>
+    <t>S026</t>
+  </si>
+  <si>
+    <t>ov:sub_vz</t>
+  </si>
+  <si>
+    <t>sub_vz</t>
+  </si>
+  <si>
+    <t>errorform</t>
+  </si>
+  <si>
+    <t>S027</t>
+  </si>
+  <si>
+    <t>ov:del_vz</t>
+  </si>
+  <si>
+    <t>del_vz</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>44-45</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>41-42</t>
+  </si>
+  <si>
+    <t>S028</t>
+  </si>
+  <si>
+    <t>ov:del_bw</t>
+  </si>
+  <si>
+    <t>del_bw</t>
+  </si>
+  <si>
+    <t>S029</t>
+  </si>
+  <si>
+    <t>ov:sub_bw</t>
+  </si>
+  <si>
+    <t>sub_bw</t>
+  </si>
+  <si>
+    <t>S030</t>
+  </si>
+  <si>
+    <t>ov:sub_vnw</t>
+  </si>
+  <si>
+    <t>sub_vnw</t>
+  </si>
+  <si>
+    <t>S031</t>
+  </si>
+  <si>
+    <t>S032</t>
+  </si>
+  <si>
+    <t>S033</t>
+  </si>
+  <si>
+    <t>ov:del_er</t>
+  </si>
+  <si>
+    <t>del_er</t>
+  </si>
+  <si>
+    <t>ov:del_vg</t>
+  </si>
+  <si>
+    <t>ov:sub_vg</t>
+  </si>
+  <si>
+    <t>sub_vg</t>
+  </si>
+  <si>
+    <t>del_vg</t>
+  </si>
+  <si>
+    <t>S034</t>
+  </si>
+  <si>
+    <t>kop weg</t>
+  </si>
+  <si>
+    <t>del_kop, kop_weg</t>
+  </si>
+  <si>
+    <t>no_copula</t>
+  </si>
+  <si>
+    <t>S035</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>verb_no_pv</t>
+  </si>
+  <si>
+    <t>S036</t>
+  </si>
+  <si>
+    <t>del_nmwg</t>
+  </si>
+  <si>
+    <t>deletie naamwrd.groep</t>
+  </si>
+  <si>
+    <t>deletie voorzetsel</t>
+  </si>
+  <si>
+    <t>deletie voegwrd</t>
+  </si>
+  <si>
+    <t>43-44</t>
+  </si>
+  <si>
+    <t>S037</t>
+  </si>
+  <si>
+    <t>adj_agreement_errors</t>
+  </si>
+  <si>
+    <t>adj_congr_fout</t>
+  </si>
+  <si>
+    <t>S038</t>
+  </si>
+  <si>
+    <t>dan_toen_fout</t>
+  </si>
+  <si>
+    <t>S039</t>
+  </si>
+  <si>
+    <t>ov:sub_tijd</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>sub_tijd</t>
+  </si>
+  <si>
+    <t>S040</t>
+  </si>
+  <si>
+    <t>hulpww weg</t>
+  </si>
+  <si>
+    <t>aux_weg, del_aux, aux weg</t>
+  </si>
+  <si>
+    <t>sub_lexicaal</t>
+  </si>
+  <si>
+    <t>sub_lexical</t>
+  </si>
+  <si>
+    <t>uitspraak_variant</t>
+  </si>
+  <si>
+    <t>S060</t>
+  </si>
+  <si>
+    <t>get_pronunciation_variants</t>
+  </si>
+  <si>
+    <t>omitted_phrase</t>
+  </si>
+  <si>
+    <t>SASTA-opmerkingen</t>
+  </si>
+  <si>
+    <t>S061</t>
+  </si>
+  <si>
+    <t>topic_drop</t>
+  </si>
+  <si>
+    <t>S062</t>
+  </si>
+  <si>
+    <t>valse_start</t>
+  </si>
+  <si>
+    <t>valse start</t>
+  </si>
+  <si>
+    <t>62-63</t>
+  </si>
+  <si>
+    <t>false_start</t>
+  </si>
+  <si>
+    <t>S063</t>
+  </si>
+  <si>
+    <t>zelfverbetering</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>self_correction</t>
+  </si>
+  <si>
+    <t>S064</t>
+  </si>
+  <si>
+    <t>herhaling</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>repetition</t>
+  </si>
+  <si>
+    <t>uitspraak-variant, uitspraakvariant, uitspraak variant</t>
+  </si>
+  <si>
+    <t>beginwoorddeletie</t>
+  </si>
+  <si>
+    <t>topic_drop, bw_del, bwd</t>
+  </si>
+  <si>
+    <t>bep deletie, bepaler_weg</t>
+  </si>
+  <si>
+    <t>S065</t>
+  </si>
+  <si>
+    <t>t_elisie</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>pv_t_elisions</t>
+  </si>
+  <si>
+    <t>t-elisie, t elisie</t>
+  </si>
+  <si>
+    <t>S041</t>
+  </si>
+  <si>
+    <t>S042</t>
+  </si>
+  <si>
+    <t>variabele 13</t>
+  </si>
+  <si>
+    <t>variabele 14</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>S043</t>
+  </si>
+  <si>
+    <t>variabele 15</t>
+  </si>
+  <si>
+    <t>vt_fout_count</t>
+  </si>
+  <si>
+    <t>congruentie_fount_count</t>
+  </si>
+  <si>
+    <t>S044</t>
+  </si>
+  <si>
+    <t>variabele 16</t>
+  </si>
+  <si>
+    <t>vd_fout_count</t>
+  </si>
+  <si>
+    <t>S045</t>
+  </si>
+  <si>
+    <t>variabele 17</t>
+  </si>
+  <si>
+    <t>nmwg_weg_count</t>
+  </si>
+  <si>
+    <t>S046</t>
+  </si>
+  <si>
+    <t>variabele 18</t>
+  </si>
+  <si>
+    <t>bepaler_weg_count</t>
+  </si>
+  <si>
+    <t>S047</t>
+  </si>
+  <si>
+    <t>variabele 19</t>
+  </si>
+  <si>
+    <t>S048</t>
+  </si>
+  <si>
+    <t>variabele 20</t>
+  </si>
+  <si>
+    <t>woordvolgordefout_count</t>
+  </si>
+  <si>
+    <t>S049</t>
+  </si>
+  <si>
+    <t>ov:uiting_count</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>congruentie_fouten_count</t>
+  </si>
+  <si>
+    <t>bepaler_verkeerd_count</t>
+  </si>
+  <si>
+    <t>ov_uiting_count</t>
+  </si>
+  <si>
+    <t>del_nmwg_count</t>
+  </si>
+  <si>
+    <t>S050</t>
+  </si>
+  <si>
+    <t>hoofdww weg</t>
+  </si>
+  <si>
+    <t>hoofdww_weg</t>
+  </si>
+  <si>
+    <t>hoofdww_weg_count</t>
+  </si>
+  <si>
+    <t>hoofdww_weg,hoofdww-weg</t>
+  </si>
+  <si>
+    <t>deletie /er/, ov:del-er</t>
+  </si>
+  <si>
+    <t>ov:sub-vg</t>
+  </si>
+  <si>
+    <t>ov:sub-tijd</t>
+  </si>
+  <si>
+    <t>sub-lexicaal</t>
+  </si>
+  <si>
+    <t>ov:sub-vnw</t>
+  </si>
+  <si>
+    <t>ov:sub-bw</t>
+  </si>
+  <si>
+    <t>ov:del-bw</t>
+  </si>
+  <si>
+    <t>ov:sub-vz</t>
+  </si>
+  <si>
+    <t>dan-toen-fout</t>
+  </si>
+  <si>
+    <t>adj-congr-fout</t>
+  </si>
+  <si>
+    <t>bbp</t>
+  </si>
+  <si>
+    <t>bbt</t>
+  </si>
+  <si>
+    <t>bbo</t>
+  </si>
+  <si>
+    <t>sociolect</t>
+  </si>
+  <si>
+    <t>taalvariatie</t>
+  </si>
+  <si>
     <t xml:space="preserve">//node[@pt="n"
     or (@pt="ww" and @positie="nom" and @rel="obj1")
     or (@pt="adj" and @positie="nom")
     or (@pt="tw" and @positie!="prenom" and (@rel!="det" and not(@rel="cnj" and parent::node[@rel="det"])))
+   or  (@pt="vnw" and @positie="nom" and @vwtype="bez")
     or (@cat="mwu") and node[@pos="name"]] 
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">//node[%STAP_OS%]
-</t>
-  </si>
-  <si>
-    <t>S020</t>
-  </si>
-  <si>
-    <t>bepaler weg</t>
-  </si>
-  <si>
-    <t>get_missing_det</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>pages2005</t>
-  </si>
-  <si>
-    <t>pages2017</t>
-  </si>
-  <si>
-    <t>acq_order</t>
-  </si>
-  <si>
-    <t>implied_by</t>
-  </si>
-  <si>
-    <t>S021</t>
-  </si>
-  <si>
-    <t>bepaler fout</t>
-  </si>
-  <si>
-    <t>grammaticale fout</t>
-  </si>
-  <si>
-    <t>S022</t>
-  </si>
-  <si>
-    <t>congruentiefout</t>
-  </si>
-  <si>
-    <t>stap_congruentiefout</t>
-  </si>
-  <si>
-    <t>S023</t>
-  </si>
-  <si>
-    <t>pv_regionale_vorm</t>
-  </si>
-  <si>
-    <t>bepalers</t>
-  </si>
-  <si>
-    <t>congruentie</t>
-  </si>
-  <si>
-    <t>S024</t>
-  </si>
-  <si>
-    <t>vt_fout</t>
-  </si>
-  <si>
-    <t>morfologie</t>
-  </si>
-  <si>
-    <t>S025</t>
-  </si>
-  <si>
-    <t>vd_fout</t>
-  </si>
-  <si>
-    <t>stap_sublid</t>
-  </si>
-  <si>
-    <t>S026</t>
-  </si>
-  <si>
-    <t>ov:sub_vz</t>
-  </si>
-  <si>
-    <t>sub_vz</t>
-  </si>
-  <si>
-    <t>errorform</t>
-  </si>
-  <si>
-    <t>S027</t>
-  </si>
-  <si>
-    <t>ov:del_vz</t>
-  </si>
-  <si>
-    <t>del_vz</t>
-  </si>
-  <si>
-    <t>46</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>44-45</t>
-  </si>
-  <si>
-    <t>43</t>
-  </si>
-  <si>
-    <t>42</t>
-  </si>
-  <si>
-    <t>41-42</t>
-  </si>
-  <si>
-    <t>S028</t>
-  </si>
-  <si>
-    <t>ov:del_bw</t>
-  </si>
-  <si>
-    <t>del_bw</t>
-  </si>
-  <si>
-    <t>S029</t>
-  </si>
-  <si>
-    <t>ov:sub_bw</t>
-  </si>
-  <si>
-    <t>sub_bw</t>
-  </si>
-  <si>
-    <t>S030</t>
-  </si>
-  <si>
-    <t>ov:sub_vnw</t>
-  </si>
-  <si>
-    <t>sub_vnw</t>
-  </si>
-  <si>
-    <t>S031</t>
-  </si>
-  <si>
-    <t>S032</t>
-  </si>
-  <si>
-    <t>S033</t>
-  </si>
-  <si>
-    <t>ov:del_er</t>
-  </si>
-  <si>
-    <t>del_er</t>
-  </si>
-  <si>
-    <t>ov:del_vg</t>
-  </si>
-  <si>
-    <t>ov:sub_vg</t>
-  </si>
-  <si>
-    <t>sub_vg</t>
-  </si>
-  <si>
-    <t>del_vg</t>
-  </si>
-  <si>
-    <t>S034</t>
-  </si>
-  <si>
-    <t>kop weg</t>
-  </si>
-  <si>
-    <t>del_kop, kop_weg</t>
-  </si>
-  <si>
-    <t>no_copula</t>
-  </si>
-  <si>
-    <t>S035</t>
-  </si>
-  <si>
-    <t>41</t>
-  </si>
-  <si>
-    <t>verb_no_pv</t>
-  </si>
-  <si>
-    <t>S036</t>
-  </si>
-  <si>
-    <t>del_nmwg</t>
-  </si>
-  <si>
-    <t>deletie naamwrd.groep</t>
-  </si>
-  <si>
-    <t>deletie voorzetsel</t>
-  </si>
-  <si>
-    <t>deletie voegwrd</t>
-  </si>
-  <si>
-    <t>43-44</t>
-  </si>
-  <si>
-    <t>S037</t>
-  </si>
-  <si>
-    <t>adj_agreement_errors</t>
-  </si>
-  <si>
-    <t>adj_congr_fout</t>
-  </si>
-  <si>
-    <t>S038</t>
-  </si>
-  <si>
-    <t>dan_toen_fout</t>
-  </si>
-  <si>
-    <t>S039</t>
-  </si>
-  <si>
-    <t>ov:sub_tijd</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>sub_tijd</t>
-  </si>
-  <si>
-    <t>S040</t>
-  </si>
-  <si>
-    <t>hulpww weg</t>
-  </si>
-  <si>
-    <t>aux_weg, del_aux, aux weg</t>
-  </si>
-  <si>
-    <t>sub_lexicaal</t>
-  </si>
-  <si>
-    <t>sub_lexical</t>
-  </si>
-  <si>
-    <t>uitspraak_variant</t>
-  </si>
-  <si>
-    <t>S060</t>
-  </si>
-  <si>
-    <t>get_pronunciation_variants</t>
-  </si>
-  <si>
-    <t>omitted_phrase</t>
-  </si>
-  <si>
-    <t>SASTA-opmerkingen</t>
-  </si>
-  <si>
-    <t>S061</t>
-  </si>
-  <si>
-    <t>topic_drop</t>
-  </si>
-  <si>
-    <t>S062</t>
-  </si>
-  <si>
-    <t>valse_start</t>
-  </si>
-  <si>
-    <t>valse start</t>
-  </si>
-  <si>
-    <t>62-63</t>
-  </si>
-  <si>
-    <t>false_start</t>
-  </si>
-  <si>
-    <t>S063</t>
-  </si>
-  <si>
-    <t>zelfverbetering</t>
-  </si>
-  <si>
-    <t>63</t>
-  </si>
-  <si>
-    <t>self_correction</t>
-  </si>
-  <si>
-    <t>S064</t>
-  </si>
-  <si>
-    <t>herhaling</t>
-  </si>
-  <si>
-    <t>64</t>
-  </si>
-  <si>
-    <t>repetition</t>
-  </si>
-  <si>
-    <t>uitspraak-variant, uitspraakvariant, uitspraak variant</t>
-  </si>
-  <si>
-    <t>beginwoorddeletie</t>
-  </si>
-  <si>
-    <t>topic_drop, bw_del, bwd</t>
-  </si>
-  <si>
-    <t>bep deletie, bepaler_weg</t>
-  </si>
-  <si>
-    <t>S065</t>
-  </si>
-  <si>
-    <t>t_elisie</t>
-  </si>
-  <si>
-    <t>none</t>
-  </si>
-  <si>
-    <t>pv_t_elisions</t>
-  </si>
-  <si>
-    <t>t-elisie, t elisie</t>
-  </si>
-  <si>
-    <t>S041</t>
-  </si>
-  <si>
-    <t>S042</t>
-  </si>
-  <si>
-    <t>variabele 13</t>
-  </si>
-  <si>
-    <t>variabele 14</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>S043</t>
-  </si>
-  <si>
-    <t>variabele 15</t>
-  </si>
-  <si>
-    <t>vt_fout_count</t>
-  </si>
-  <si>
-    <t>congruentie_fount_count</t>
-  </si>
-  <si>
-    <t>S044</t>
-  </si>
-  <si>
-    <t>variabele 16</t>
-  </si>
-  <si>
-    <t>vd_fout_count</t>
-  </si>
-  <si>
-    <t>S045</t>
-  </si>
-  <si>
-    <t>variabele 17</t>
-  </si>
-  <si>
-    <t>nmwg_weg_count</t>
-  </si>
-  <si>
-    <t>S046</t>
-  </si>
-  <si>
-    <t>variabele 18</t>
-  </si>
-  <si>
-    <t>bepaler_weg_count</t>
-  </si>
-  <si>
-    <t>S047</t>
-  </si>
-  <si>
-    <t>variabele 19</t>
-  </si>
-  <si>
-    <t>S048</t>
-  </si>
-  <si>
-    <t>variabele 20</t>
-  </si>
-  <si>
-    <t>woordvolgordefout_count</t>
-  </si>
-  <si>
-    <t>S049</t>
-  </si>
-  <si>
-    <t>ov:uiting_count</t>
-  </si>
-  <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>congruentie_fouten_count</t>
-  </si>
-  <si>
-    <t>bepaler_verkeerd_count</t>
-  </si>
-  <si>
-    <t>ov_uiting_count</t>
-  </si>
-  <si>
-    <t>del_nmwg_count</t>
-  </si>
-  <si>
-    <t>S050</t>
-  </si>
-  <si>
-    <t>hoofdww weg</t>
-  </si>
-  <si>
-    <t>hoofdww_weg</t>
-  </si>
-  <si>
-    <t>hoofdww_weg_count</t>
-  </si>
-  <si>
-    <t>hoofdww_weg,hoofdww-weg</t>
-  </si>
-  <si>
-    <t>deletie /er/, ov:del-er</t>
-  </si>
-  <si>
-    <t>ov:sub-vg</t>
-  </si>
-  <si>
-    <t>ov:sub-tijd</t>
-  </si>
-  <si>
-    <t>sub-lexicaal</t>
-  </si>
-  <si>
-    <t>ov:sub-vnw</t>
-  </si>
-  <si>
-    <t>ov:sub-bw</t>
-  </si>
-  <si>
-    <t>ov:del-bw</t>
-  </si>
-  <si>
-    <t>ov:sub-vz</t>
-  </si>
-  <si>
-    <t>dan-toen-fout</t>
-  </si>
-  <si>
-    <t>adj-congr-fout</t>
-  </si>
-  <si>
-    <t>bbp</t>
-  </si>
-  <si>
-    <t>bbt</t>
-  </si>
-  <si>
-    <t>bbo</t>
-  </si>
-  <si>
-    <t>sociolect</t>
-  </si>
-  <si>
-    <t>taalvariatie</t>
   </si>
 </sst>
 </file>
@@ -1526,10 +1527,10 @@
         <v>11</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>3</v>
@@ -1559,10 +1560,10 @@
         <v>147</v>
       </c>
       <c r="T1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>162</v>
       </c>
       <c r="V1" s="1" t="s">
         <v>148</v>
@@ -1638,7 +1639,7 @@
         <v>96</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>97</v>
@@ -1805,7 +1806,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:24" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>42</v>
       </c>
@@ -1831,7 +1832,7 @@
         <v>96</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>153</v>
+        <v>316</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>97</v>
@@ -1942,7 +1943,7 @@
         <v>93</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>97</v>
@@ -1983,7 +1984,7 @@
         <v>89</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>97</v>
@@ -2024,7 +2025,7 @@
         <v>83</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>97</v>
@@ -2302,547 +2303,547 @@
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E21" s="2" t="s">
+      <c r="F21" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="L21" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>157</v>
-      </c>
       <c r="M21" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O21" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X21" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>164</v>
-      </c>
       <c r="H22" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O22" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X22" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E23" s="2" t="s">
+      <c r="H23" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="L23" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="H23" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>168</v>
-      </c>
       <c r="M23" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X23" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>97</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O24" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X24" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="H25" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O25" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X25" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>177</v>
-      </c>
       <c r="H26" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O26" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X26" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E27" s="2" t="s">
+      <c r="F27" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="L27" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="F27" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="L27" s="2" t="s">
+      <c r="M27" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="M27" s="2" t="s">
-        <v>182</v>
-      </c>
       <c r="N27" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O27" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X27" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E28" s="2" t="s">
+      <c r="F28" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="L28" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>185</v>
-      </c>
       <c r="M28" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O28" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X28" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E29" s="2" t="s">
+      <c r="F29" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="L29" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="F29" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="L29" s="2" t="s">
-        <v>194</v>
-      </c>
       <c r="M29" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O29" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X29" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E30" s="2" t="s">
+      <c r="F30" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="L30" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>197</v>
-      </c>
       <c r="M30" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O30" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X30" s="2" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E31" s="2" t="s">
+      <c r="F31" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="L31" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="F31" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>200</v>
-      </c>
       <c r="M31" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O31" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X31" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O32" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X32" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="33" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E33" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="L33" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="F33" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="L33" s="2" t="s">
-        <v>208</v>
-      </c>
       <c r="M33" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O33" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X33" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E34" s="2" t="s">
+      <c r="F34" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="L34" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I34" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>205</v>
-      </c>
       <c r="M34" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O34" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X34" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="35" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E35" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="H35" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="L35" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="H35" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>213</v>
-      </c>
       <c r="M35" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O35" s="2" t="s">
         <v>104</v>
       </c>
       <c r="X35" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I36" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I36" s="2" t="s">
+      <c r="L36" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="L36" s="2" t="s">
-        <v>216</v>
-      </c>
       <c r="M36" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O36" s="2" t="s">
         <v>104</v>
@@ -2850,31 +2851,31 @@
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="D37" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E37" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F37" s="2" t="s">
-        <v>219</v>
-      </c>
       <c r="H37" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O37" s="2" t="s">
         <v>104</v>
@@ -2882,31 +2883,31 @@
     </row>
     <row r="38" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="L38" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="L38" s="2" t="s">
-        <v>224</v>
-      </c>
       <c r="M38" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O38" s="2" t="s">
         <v>104</v>
@@ -2914,28 +2915,28 @@
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E39" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>227</v>
-      </c>
       <c r="F39" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>97</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O39" s="2" t="s">
         <v>104</v>
@@ -2943,31 +2944,31 @@
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E40" s="2" t="s">
+      <c r="F40" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I40" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="F40" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I40" s="2" t="s">
+      <c r="L40" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="L40" s="2" t="s">
-        <v>231</v>
-      </c>
       <c r="M40" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O40" s="2" t="s">
         <v>104</v>
@@ -2975,28 +2976,28 @@
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E41" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="L41" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="F41" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>236</v>
-      </c>
       <c r="M41" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O41" s="2" t="s">
         <v>104</v>
@@ -3004,31 +3005,31 @@
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O42" s="2" t="s">
         <v>108</v>
@@ -3036,31 +3037,31 @@
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I43" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I43" s="2" t="s">
-        <v>270</v>
-      </c>
       <c r="L43" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O43" s="2" t="s">
         <v>108</v>
@@ -3068,31 +3069,31 @@
     </row>
     <row r="44" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="D44" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>273</v>
-      </c>
       <c r="H44" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O44" s="2" t="s">
         <v>108</v>
@@ -3100,31 +3101,31 @@
     </row>
     <row r="45" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="D45" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>277</v>
-      </c>
       <c r="H45" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O45" s="2" t="s">
         <v>108</v>
@@ -3132,31 +3133,31 @@
     </row>
     <row r="46" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="D46" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E46" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>280</v>
-      </c>
       <c r="H46" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O46" s="2" t="s">
         <v>108</v>
@@ -3164,31 +3165,31 @@
     </row>
     <row r="47" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="D47" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E47" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="D47" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>283</v>
-      </c>
       <c r="H47" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O47" s="2" t="s">
         <v>108</v>
@@ -3196,31 +3197,31 @@
     </row>
     <row r="48" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>285</v>
-      </c>
       <c r="D48" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O48" s="2" t="s">
         <v>108</v>
@@ -3228,29 +3229,29 @@
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="D49" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E49" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>288</v>
-      </c>
       <c r="H49" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="L49" s="2"/>
       <c r="M49" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O49" s="2" t="s">
         <v>108</v>
@@ -3258,28 +3259,28 @@
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E50" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>290</v>
-      </c>
       <c r="H50" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O50" s="2" t="s">
         <v>108</v>
@@ -3287,31 +3288,31 @@
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E51" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="D51" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E51" s="2" t="s">
+      <c r="F51" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="L51" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="F51" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="H51" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I51" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="L51" s="2" t="s">
-        <v>299</v>
-      </c>
       <c r="M51" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O51" s="2" t="s">
         <v>104</v>
@@ -3319,28 +3320,28 @@
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="L52" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="D52" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="L52" s="2" t="s">
-        <v>239</v>
-      </c>
       <c r="M52" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O52" s="2" t="s">
         <v>104</v>
@@ -3348,28 +3349,28 @@
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="L53" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="D53" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="H53" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="L53" s="2" t="s">
-        <v>243</v>
-      </c>
       <c r="M53" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O53" s="2" t="s">
         <v>104</v>
@@ -3377,31 +3378,31 @@
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E54" s="2" t="s">
+      <c r="F54" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="F54" s="2" t="s">
+      <c r="H54" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I54" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="H54" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I54" s="2" t="s">
+      <c r="L54" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="L54" s="2" t="s">
-        <v>248</v>
-      </c>
       <c r="M54" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O54" s="2" t="s">
         <v>104</v>
@@ -3409,28 +3410,28 @@
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E55" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="D55" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E55" s="2" t="s">
+      <c r="H55" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I55" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="H55" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I55" s="2" t="s">
+      <c r="L55" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="L55" s="2" t="s">
-        <v>252</v>
-      </c>
       <c r="M55" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O55" s="2" t="s">
         <v>104</v>
@@ -3438,28 +3439,28 @@
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E56" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E56" s="2" t="s">
+      <c r="H56" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I56" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="H56" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I56" s="2" t="s">
+      <c r="L56" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="L56" s="2" t="s">
-        <v>256</v>
-      </c>
       <c r="M56" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O56" s="2" t="s">
         <v>104</v>
@@ -3467,31 +3468,31 @@
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E57" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E57" s="2" t="s">
+      <c r="F57" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I57" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="F57" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="H57" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="I57" s="2" t="s">
+      <c r="L57" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="L57" s="2" t="s">
-        <v>264</v>
-      </c>
       <c r="M57" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O57" s="2" t="s">
         <v>104</v>

</xml_diff>